<commit_message>
refactor(eckr): relabel Cone -> Metal Shade Pendant Light, 5 sold-proven competitors
Per Jarsini: renamed the Cone category to Metal Shade Pendant Light and
re-scraped that term (27 sold-visible) for 5 sold-proven competitors incl.
new sellers homeessenceltd, buybox786. Spider kept as-is (already has many).
Now 44 rows, all with sold history.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_SOLD.xlsx
+++ b/development/abiraj_mini_aios_workbench/projects/PRJ-2026-017_ebay-competitor-keyword-research/evidence/final_outputs/REQ-20_ebay-competitor-keyword-research/REQ-20-D01_ebay_competitor_keyword_SOLD.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N43"/>
+  <dimension ref="A1:N45"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -522,7 +522,7 @@
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Cone metal pendantlight</t>
+          <t>Metal Shade Pendant Light</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
@@ -532,32 +532,32 @@
       </c>
       <c r="C2" s="2" t="inlineStr">
         <is>
-          <t>352999718430</t>
+          <t>333675680799</t>
         </is>
       </c>
       <c r="D2" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
         <is>
-          <t>Easy Fit Lampshade Traditional Frosted Alabaster Glass Pendant</t>
+          <t>Set of 2 Modern Three Tier Easy Fit Jewelled Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>2,392</t>
+          <t>751</t>
         </is>
       </c>
       <c r="G2" s="2" t="inlineStr">
         <is>
-          <t>GBP 18.99</t>
+          <t>GBP 20.39</t>
         </is>
       </c>
       <c r="H2" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I2" s="2" t="inlineStr">
@@ -567,27 +567,27 @@
       </c>
       <c r="J2" s="2" t="inlineStr">
         <is>
-          <t>10% off</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K2" s="2" t="inlineStr">
         <is>
-          <t>Cone Pendant Light, Metal Pendant Light, Hanging Ceiling Light</t>
+          <t>Metal Shade Pendant Light, Metal Pendant Light, Hanging Pendant Light</t>
         </is>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Pendant, Industrial Pendant Light, Kitchen Pendant, Retro Hanging Light</t>
+          <t>Ceiling Pendant Shade, Industrial Pendant Light, Easy Fit Pendant Shade, Kitchen Pendant Light</t>
         </is>
       </c>
       <c r="M2" s="2" t="inlineStr">
         <is>
-          <t>Black Metal Cone Pendant Light for Kitchen Island, Adjustable Industrial Ceiling Pendant E27, Vintage Cone Hanging Lamp for Dining Room</t>
+          <t>Black Metal Shade Pendant Light for Kitchen Island, Industrial Easy Fit Metal Pendant Shade E27, Modern Chrome Metal Pendant Ceiling Light</t>
         </is>
       </c>
       <c r="N2" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: firstchoicelightingoutlet.</t>
         </is>
       </c>
     </row>
@@ -596,32 +596,32 @@
       <c r="B3" s="2" t="inlineStr"/>
       <c r="C3" s="2" t="inlineStr">
         <is>
-          <t>352643317600</t>
+          <t>285423964421</t>
         </is>
       </c>
       <c r="D3" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Giggi</t>
         </is>
       </c>
       <c r="E3" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Shade Modern Tapered Frosted Glass Pendant Lamp</t>
+          <t>Metal &amp; Rope Lamp Shades Ceiling Pendant Light Shade</t>
         </is>
       </c>
       <c r="F3" s="2" t="inlineStr">
         <is>
-          <t>1,863</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G3" s="2" t="inlineStr">
         <is>
-          <t>GBP 17.99</t>
+          <t>GBP 18.99</t>
         </is>
       </c>
       <c r="H3" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.6% (21.9K)</t>
         </is>
       </c>
       <c r="I3" s="2" t="inlineStr">
@@ -631,7 +631,7 @@
       </c>
       <c r="J3" s="2" t="inlineStr">
         <is>
-          <t>10% off</t>
+          <t>Save up to 15% Multi-buy</t>
         </is>
       </c>
       <c r="K3" s="2" t="inlineStr"/>
@@ -639,7 +639,7 @@
       <c r="M3" s="2" t="inlineStr"/>
       <c r="N3" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: picknmix.online.</t>
         </is>
       </c>
     </row>
@@ -648,32 +648,32 @@
       <c r="B4" s="2" t="inlineStr"/>
       <c r="C4" s="2" t="inlineStr">
         <is>
-          <t>131168385082</t>
+          <t>372257187156</t>
         </is>
       </c>
       <c r="D4" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
         <is>
-          <t>Clear Well Glass Light Shade Cylinder Replacement Pendant Shade</t>
+          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl Glass</t>
         </is>
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>51</t>
+          <t>8,367</t>
         </is>
       </c>
       <c r="G4" s="2" t="inlineStr">
         <is>
-          <t>GBP 38.08</t>
+          <t>GBP 19.99</t>
         </is>
       </c>
       <c r="H4" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I4" s="2" t="inlineStr">
@@ -691,45 +691,41 @@
       <c r="M4" s="2" t="inlineStr"/>
       <c r="N4" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="inlineStr">
-        <is>
-          <t>Wall Light</t>
-        </is>
-      </c>
+      <c r="A5" s="2" t="inlineStr"/>
       <c r="B5" s="2" t="inlineStr"/>
       <c r="C5" s="2" t="inlineStr">
         <is>
-          <t>115699570601</t>
+          <t>154695326074</t>
         </is>
       </c>
       <c r="D5" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>Innoteck</t>
         </is>
       </c>
       <c r="E5" s="2" t="inlineStr">
         <is>
-          <t>Vintage Industrial Wall Light Antique Retro Cage Bulkhead Gold Brass Ship Lamp</t>
+          <t>Ceiling Light Shade Chandelier Pendant Acrylic Crystal Droplet Chrome</t>
         </is>
       </c>
       <c r="F5" s="2" t="inlineStr">
         <is>
-          <t>257</t>
+          <t>354+</t>
         </is>
       </c>
       <c r="G5" s="2" t="inlineStr">
         <is>
-          <t>GBP 64.99</t>
+          <t>GBP 10.99</t>
         </is>
       </c>
       <c r="H5" s="2" t="inlineStr">
         <is>
-          <t>100% (1.4K)</t>
+          <t>99.9% (60.1K)</t>
         </is>
       </c>
       <c r="I5" s="2" t="inlineStr">
@@ -739,27 +735,15 @@
       </c>
       <c r="J5" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K5" s="2" t="inlineStr">
-        <is>
-          <t>Wall Light, Wall Lamp, Wall Sconce</t>
-        </is>
-      </c>
-      <c r="L5" s="2" t="inlineStr">
-        <is>
-          <t>Indoor Wall Light, Bedside Wall Lamp, Industrial Wall Sconce, LED Wall Light</t>
-        </is>
-      </c>
-      <c r="M5" s="2" t="inlineStr">
-        <is>
-          <t>Black Industrial Wall Light for Living Room, Vintage Wall Sconce with Switch, Modern LED Bedside Wall Reading Lamp</t>
-        </is>
-      </c>
+          <t>Save up to 20% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K5" s="2" t="inlineStr"/>
+      <c r="L5" s="2" t="inlineStr"/>
+      <c r="M5" s="2" t="inlineStr"/>
       <c r="N5" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: eat_sleep_buy_repeat.</t>
+          <t>Competitor seller: homeessenceltd.</t>
         </is>
       </c>
     </row>
@@ -768,32 +752,32 @@
       <c r="B6" s="2" t="inlineStr"/>
       <c r="C6" s="2" t="inlineStr">
         <is>
-          <t>234566652967</t>
+          <t>201620721277</t>
         </is>
       </c>
       <c r="D6" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>OPTIMAL PRODUCTS</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>Vintage Industrial Wall Light Antique Retro Style Lamp Sconce Fixture Rustic</t>
+          <t>Chandelier Style Ceiling Light Shade Droplet Pendant Acrylic Crystal Bead</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>71</t>
+          <t>65+</t>
         </is>
       </c>
       <c r="G6" s="2" t="inlineStr">
         <is>
-          <t>GBP 31.99</t>
+          <t>GBP 10.95 to 19.95</t>
         </is>
       </c>
       <c r="H6" s="2" t="inlineStr">
         <is>
-          <t>99.7% (9.8K)</t>
+          <t>99.7% (220.4K)</t>
         </is>
       </c>
       <c r="I6" s="2" t="inlineStr">
@@ -803,7 +787,7 @@
       </c>
       <c r="J6" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Save up to 6% Multi-buy</t>
         </is>
       </c>
       <c r="K6" s="2" t="inlineStr"/>
@@ -811,41 +795,45 @@
       <c r="M6" s="2" t="inlineStr"/>
       <c r="N6" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: burgesshandg.</t>
+          <t>Competitor seller: buybox786.</t>
         </is>
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="inlineStr"/>
+      <c r="A7" s="2" t="inlineStr">
+        <is>
+          <t>Wall Light</t>
+        </is>
+      </c>
       <c r="B7" s="2" t="inlineStr"/>
       <c r="C7" s="2" t="inlineStr">
         <is>
-          <t>155030374927</t>
+          <t>115699570601</t>
         </is>
       </c>
       <c r="D7" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E7" s="2" t="inlineStr">
         <is>
-          <t>Modern Vintage Retro Industrial Rustic Sconce Wall Light</t>
+          <t>Vintage Industrial Wall Light Antique Retro Cage Bulkhead Gold Brass Ship Lamp</t>
         </is>
       </c>
       <c r="F7" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>257</t>
         </is>
       </c>
       <c r="G7" s="2" t="inlineStr">
         <is>
-          <t>GBP 7.99</t>
+          <t>GBP 64.99</t>
         </is>
       </c>
       <c r="H7" s="2" t="inlineStr">
         <is>
-          <t>99.7% (5.5K)</t>
+          <t>100% (1.4K)</t>
         </is>
       </c>
       <c r="I7" s="2" t="inlineStr">
@@ -855,15 +843,27 @@
       </c>
       <c r="J7" s="2" t="inlineStr">
         <is>
-          <t>Save up to 6% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K7" s="2" t="inlineStr"/>
-      <c r="L7" s="2" t="inlineStr"/>
-      <c r="M7" s="2" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K7" s="2" t="inlineStr">
+        <is>
+          <t>Wall Light, Wall Lamp, Wall Sconce</t>
+        </is>
+      </c>
+      <c r="L7" s="2" t="inlineStr">
+        <is>
+          <t>Indoor Wall Light, Bedside Wall Lamp, Industrial Wall Sconce, LED Wall Light</t>
+        </is>
+      </c>
+      <c r="M7" s="2" t="inlineStr">
+        <is>
+          <t>Black Industrial Wall Light for Living Room, Vintage Wall Sconce with Switch, Modern LED Bedside Wall Reading Lamp</t>
+        </is>
+      </c>
       <c r="N7" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: theyinltd.</t>
+          <t>Competitor seller: eat_sleep_buy_repeat.</t>
         </is>
       </c>
     </row>
@@ -872,7 +872,7 @@
       <c r="B8" s="2" t="inlineStr"/>
       <c r="C8" s="2" t="inlineStr">
         <is>
-          <t>116478119802</t>
+          <t>234566652967</t>
         </is>
       </c>
       <c r="D8" s="2" t="inlineStr">
@@ -882,22 +882,22 @@
       </c>
       <c r="E8" s="2" t="inlineStr">
         <is>
-          <t>Industrial Bulkhead Light Wall Ceiling Retro Old Marine Brass Gold</t>
+          <t>Vintage Industrial Wall Light Antique Retro Style Lamp Sconce Fixture Rustic</t>
         </is>
       </c>
       <c r="F8" s="2" t="inlineStr">
         <is>
-          <t>61</t>
+          <t>71</t>
         </is>
       </c>
       <c r="G8" s="2" t="inlineStr">
         <is>
-          <t>GBP 69.99</t>
+          <t>GBP 31.99</t>
         </is>
       </c>
       <c r="H8" s="2" t="inlineStr">
         <is>
-          <t>100% (1.4K)</t>
+          <t>99.7% (9.8K)</t>
         </is>
       </c>
       <c r="I8" s="2" t="inlineStr">
@@ -915,7 +915,7 @@
       <c r="M8" s="2" t="inlineStr"/>
       <c r="N8" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: eat_sleep_buy_repeat.</t>
+          <t>Competitor seller: burgesshandg.</t>
         </is>
       </c>
     </row>
@@ -924,32 +924,32 @@
       <c r="B9" s="2" t="inlineStr"/>
       <c r="C9" s="2" t="inlineStr">
         <is>
-          <t>137354830445</t>
+          <t>155030374927</t>
         </is>
       </c>
       <c r="D9" s="2" t="inlineStr">
         <is>
-          <t>Does not apply</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E9" s="2" t="inlineStr">
         <is>
-          <t>Vintage Brass Boho Wall Sconces with Tulip Glass Shade for Modern Spaces</t>
+          <t>Modern Vintage Retro Industrial Rustic Sconce Wall Light</t>
         </is>
       </c>
       <c r="F9" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>61</t>
         </is>
       </c>
       <c r="G9" s="2" t="inlineStr">
         <is>
-          <t>GBP 81.26</t>
+          <t>GBP 7.99</t>
         </is>
       </c>
       <c r="H9" s="2" t="inlineStr">
         <is>
-          <t>99.8% (28.1K)</t>
+          <t>99.7% (5.5K)</t>
         </is>
       </c>
       <c r="I9" s="2" t="inlineStr">
@@ -959,7 +959,7 @@
       </c>
       <c r="J9" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Save up to 6% Multi-buy</t>
         </is>
       </c>
       <c r="K9" s="2" t="inlineStr"/>
@@ -967,45 +967,41 @@
       <c r="M9" s="2" t="inlineStr"/>
       <c r="N9" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: weshipnow.</t>
+          <t>Competitor seller: theyinltd.</t>
         </is>
       </c>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="inlineStr">
-        <is>
-          <t>Metal shade Ceiling Light</t>
-        </is>
-      </c>
+      <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="2" t="inlineStr"/>
       <c r="C10" s="2" t="inlineStr">
         <is>
-          <t>372257187156</t>
+          <t>116478119802</t>
         </is>
       </c>
       <c r="D10" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E10" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl Glass</t>
+          <t>Industrial Bulkhead Light Wall Ceiling Retro Old Marine Brass Gold</t>
         </is>
       </c>
       <c r="F10" s="2" t="inlineStr">
         <is>
-          <t>8,367</t>
+          <t>61</t>
         </is>
       </c>
       <c r="G10" s="2" t="inlineStr">
         <is>
-          <t>GBP 19.99</t>
+          <t>GBP 69.99</t>
         </is>
       </c>
       <c r="H10" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>100% (1.4K)</t>
         </is>
       </c>
       <c r="I10" s="2" t="inlineStr">
@@ -1018,24 +1014,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K10" s="2" t="inlineStr">
-        <is>
-          <t>Metal Ceiling Light, Ceiling Shade, Metal Pendant Shade</t>
-        </is>
-      </c>
-      <c r="L10" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Ceiling Light, Metal Lampshade, Ceiling Light Fitting, Retro Ceiling Shade</t>
-        </is>
-      </c>
-      <c r="M10" s="2" t="inlineStr">
-        <is>
-          <t>Black Metal Ceiling Light Shade for Kitchen, Industrial Metal Pendant Shade E27, Vintage Metal Ceiling Lampshade Easy Fit</t>
-        </is>
-      </c>
+      <c r="K10" s="2" t="inlineStr"/>
+      <c r="L10" s="2" t="inlineStr"/>
+      <c r="M10" s="2" t="inlineStr"/>
       <c r="N10" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: eat_sleep_buy_repeat.</t>
         </is>
       </c>
     </row>
@@ -1044,32 +1028,32 @@
       <c r="B11" s="2" t="inlineStr"/>
       <c r="C11" s="2" t="inlineStr">
         <is>
-          <t>372336415252</t>
+          <t>137354830445</t>
         </is>
       </c>
       <c r="D11" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Does not apply</t>
         </is>
       </c>
       <c r="E11" s="2" t="inlineStr">
         <is>
-          <t>Lampshade Ceiling Pendant Light Shade Easy Fit Chandelier</t>
+          <t>Vintage Brass Boho Wall Sconces with Tulip Glass Shade for Modern Spaces</t>
         </is>
       </c>
       <c r="F11" s="2" t="inlineStr">
         <is>
-          <t>6,442+</t>
+          <t>2</t>
         </is>
       </c>
       <c r="G11" s="2" t="inlineStr">
         <is>
-          <t>GBP 17.99</t>
+          <t>GBP 81.26</t>
         </is>
       </c>
       <c r="H11" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.8% (28.1K)</t>
         </is>
       </c>
       <c r="I11" s="2" t="inlineStr">
@@ -1079,7 +1063,7 @@
       </c>
       <c r="J11" s="2" t="inlineStr">
         <is>
-          <t>Save up to 10% Multi-buy</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K11" s="2" t="inlineStr"/>
@@ -1087,41 +1071,45 @@
       <c r="M11" s="2" t="inlineStr"/>
       <c r="N11" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: weshipnow.</t>
         </is>
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="inlineStr"/>
+      <c r="A12" s="2" t="inlineStr">
+        <is>
+          <t>Metal shade Ceiling Light</t>
+        </is>
+      </c>
       <c r="B12" s="2" t="inlineStr"/>
       <c r="C12" s="2" t="inlineStr">
         <is>
-          <t>333667118358</t>
+          <t>372257187156</t>
         </is>
       </c>
       <c r="D12" s="2" t="inlineStr">
         <is>
-          <t>firstchoicelighting</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E12" s="2" t="inlineStr">
         <is>
-          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
+          <t>Ceiling Light Fitting 3 Way Chrome Spotlight Swirl Glass</t>
         </is>
       </c>
       <c r="F12" s="2" t="inlineStr">
         <is>
-          <t>268</t>
+          <t>8,367</t>
         </is>
       </c>
       <c r="G12" s="2" t="inlineStr">
         <is>
-          <t>GBP 23.45</t>
+          <t>GBP 19.99</t>
         </is>
       </c>
       <c r="H12" s="2" t="inlineStr">
         <is>
-          <t>99.7% (89.9K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I12" s="2" t="inlineStr">
@@ -1134,12 +1122,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K12" s="2" t="inlineStr"/>
-      <c r="L12" s="2" t="inlineStr"/>
-      <c r="M12" s="2" t="inlineStr"/>
+      <c r="K12" s="2" t="inlineStr">
+        <is>
+          <t>Metal Ceiling Light, Ceiling Shade, Metal Pendant Shade</t>
+        </is>
+      </c>
+      <c r="L12" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Ceiling Light, Metal Lampshade, Ceiling Light Fitting, Retro Ceiling Shade</t>
+        </is>
+      </c>
+      <c r="M12" s="2" t="inlineStr">
+        <is>
+          <t>Black Metal Ceiling Light Shade for Kitchen, Industrial Metal Pendant Shade E27, Vintage Metal Ceiling Lampshade Easy Fit</t>
+        </is>
+      </c>
       <c r="N12" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: firstchoicelightingoutlet.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
@@ -1148,32 +1148,32 @@
       <c r="B13" s="2" t="inlineStr"/>
       <c r="C13" s="2" t="inlineStr">
         <is>
-          <t>285423964421</t>
+          <t>372336415252</t>
         </is>
       </c>
       <c r="D13" s="2" t="inlineStr">
         <is>
-          <t>Giggi</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E13" s="2" t="inlineStr">
         <is>
-          <t>Metal &amp; Rope Lamp Shades Ceiling Pendant Light Shade</t>
+          <t>Lampshade Ceiling Pendant Light Shade Easy Fit Chandelier</t>
         </is>
       </c>
       <c r="F13" s="2" t="inlineStr">
         <is>
-          <t>236</t>
+          <t>6,442+</t>
         </is>
       </c>
       <c r="G13" s="2" t="inlineStr">
         <is>
-          <t>GBP 18.99</t>
+          <t>GBP 17.99</t>
         </is>
       </c>
       <c r="H13" s="2" t="inlineStr">
         <is>
-          <t>99.6% (21.9K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I13" s="2" t="inlineStr">
@@ -1183,7 +1183,7 @@
       </c>
       <c r="J13" s="2" t="inlineStr">
         <is>
-          <t>Save up to 15% Multi-buy</t>
+          <t>Save up to 10% Multi-buy</t>
         </is>
       </c>
       <c r="K13" s="2" t="inlineStr"/>
@@ -1191,7 +1191,7 @@
       <c r="M13" s="2" t="inlineStr"/>
       <c r="N13" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: picknmix.online.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
@@ -1200,32 +1200,32 @@
       <c r="B14" s="2" t="inlineStr"/>
       <c r="C14" s="2" t="inlineStr">
         <is>
-          <t>393696656791</t>
+          <t>333667118358</t>
         </is>
       </c>
       <c r="D14" s="2" t="inlineStr">
         <is>
-          <t>Innoteck</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E14" s="2" t="inlineStr">
         <is>
-          <t>Innoteck Ceiling Light Shade - Modern Chandelier Pendant</t>
+          <t>Set of 2 Modern Black Metal Swirl Easy Fit Ceiling Light Shade</t>
         </is>
       </c>
       <c r="F14" s="2" t="inlineStr">
         <is>
-          <t>92+</t>
+          <t>268</t>
         </is>
       </c>
       <c r="G14" s="2" t="inlineStr">
         <is>
-          <t>GBP 10.49</t>
+          <t>GBP 23.45</t>
         </is>
       </c>
       <c r="H14" s="2" t="inlineStr">
         <is>
-          <t>99.8% (10.2K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I14" s="2" t="inlineStr">
@@ -1235,7 +1235,7 @@
       </c>
       <c r="J14" s="2" t="inlineStr">
         <is>
-          <t>Save up to 20% Multi-buy</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K14" s="2" t="inlineStr"/>
@@ -1243,45 +1243,41 @@
       <c r="M14" s="2" t="inlineStr"/>
       <c r="N14" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: innoteck_uk.</t>
+          <t>Competitor seller: firstchoicelightingoutlet.</t>
         </is>
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="inlineStr">
-        <is>
-          <t>Glass shade ceiling light</t>
-        </is>
-      </c>
+      <c r="A15" s="2" t="inlineStr"/>
       <c r="B15" s="2" t="inlineStr"/>
       <c r="C15" s="2" t="inlineStr">
         <is>
-          <t>333675680799</t>
+          <t>285423964421</t>
         </is>
       </c>
       <c r="D15" s="2" t="inlineStr">
         <is>
-          <t>firstchoicelighting</t>
+          <t>Giggi</t>
         </is>
       </c>
       <c r="E15" s="2" t="inlineStr">
         <is>
-          <t>Set of 2 Modern Three Tier Easy Fit Jewelled Ceiling Light</t>
+          <t>Metal &amp; Rope Lamp Shades Ceiling Pendant Light Shade</t>
         </is>
       </c>
       <c r="F15" s="2" t="inlineStr">
         <is>
-          <t>751</t>
+          <t>236</t>
         </is>
       </c>
       <c r="G15" s="2" t="inlineStr">
         <is>
-          <t>GBP 20.39</t>
+          <t>GBP 18.99</t>
         </is>
       </c>
       <c r="H15" s="2" t="inlineStr">
         <is>
-          <t>99.7% (89.9K)</t>
+          <t>99.6% (21.9K)</t>
         </is>
       </c>
       <c r="I15" s="2" t="inlineStr">
@@ -1291,27 +1287,15 @@
       </c>
       <c r="J15" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K15" s="2" t="inlineStr">
-        <is>
-          <t>Glass Ceiling Light, Glass Pendant Light, Glass Shade</t>
-        </is>
-      </c>
-      <c r="L15" s="2" t="inlineStr">
-        <is>
-          <t>Clear Glass Pendant, Glass Lampshade, Ceiling Glass Light Fitting, Modern Glass Pendant</t>
-        </is>
-      </c>
-      <c r="M15" s="2" t="inlineStr">
-        <is>
-          <t>Clear Glass Globe Pendant Light for Kitchen Island, Vintage Glass Ceiling Shade E27, Modern Frosted Glass Hanging Light</t>
-        </is>
-      </c>
+          <t>Save up to 15% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K15" s="2" t="inlineStr"/>
+      <c r="L15" s="2" t="inlineStr"/>
+      <c r="M15" s="2" t="inlineStr"/>
       <c r="N15" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: firstchoicelightingoutlet.</t>
+          <t>Competitor seller: picknmix.online.</t>
         </is>
       </c>
     </row>
@@ -1320,32 +1304,32 @@
       <c r="B16" s="2" t="inlineStr"/>
       <c r="C16" s="2" t="inlineStr">
         <is>
-          <t>283064879219</t>
+          <t>393696656791</t>
         </is>
       </c>
       <c r="D16" s="2" t="inlineStr">
         <is>
-          <t>Giggi</t>
+          <t>Innoteck</t>
         </is>
       </c>
       <c r="E16" s="2" t="inlineStr">
         <is>
-          <t>Modern Chandelier Style Ceiling Pendant Light Shade K9</t>
+          <t>Innoteck Ceiling Light Shade - Modern Chandelier Pendant</t>
         </is>
       </c>
       <c r="F16" s="2" t="inlineStr">
         <is>
-          <t>600</t>
+          <t>92+</t>
         </is>
       </c>
       <c r="G16" s="2" t="inlineStr">
         <is>
-          <t>GBP 21.99</t>
+          <t>GBP 10.49</t>
         </is>
       </c>
       <c r="H16" s="2" t="inlineStr">
         <is>
-          <t>99.6% (21.9K)</t>
+          <t>99.8% (10.2K)</t>
         </is>
       </c>
       <c r="I16" s="2" t="inlineStr">
@@ -1355,7 +1339,7 @@
       </c>
       <c r="J16" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Save up to 20% Multi-buy</t>
         </is>
       </c>
       <c r="K16" s="2" t="inlineStr"/>
@@ -1363,41 +1347,45 @@
       <c r="M16" s="2" t="inlineStr"/>
       <c r="N16" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: picknmix.online.</t>
+          <t>Competitor seller: innoteck_uk.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="inlineStr"/>
+      <c r="A17" s="2" t="inlineStr">
+        <is>
+          <t>Glass shade ceiling light</t>
+        </is>
+      </c>
       <c r="B17" s="2" t="inlineStr"/>
       <c r="C17" s="2" t="inlineStr">
         <is>
-          <t>272110237788</t>
+          <t>333675680799</t>
         </is>
       </c>
       <c r="D17" s="2" t="inlineStr">
         <is>
-          <t>MoonLight Retail</t>
+          <t>firstchoicelighting</t>
         </is>
       </c>
       <c r="E17" s="2" t="inlineStr">
         <is>
-          <t>New Modern Vintage Industrial Retro Loft Glass Ceiling Lamp Shade</t>
+          <t>Set of 2 Modern Three Tier Easy Fit Jewelled Ceiling Light</t>
         </is>
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t>269+</t>
+          <t>751</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>GBP 32.47 to 35.83</t>
+          <t>GBP 20.39</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t>100% (3.9K)</t>
+          <t>99.7% (89.9K)</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -1407,15 +1395,27 @@
       </c>
       <c r="J17" s="2" t="inlineStr">
         <is>
-          <t>Save up to 5% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K17" s="2" t="inlineStr"/>
-      <c r="L17" s="2" t="inlineStr"/>
-      <c r="M17" s="2" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K17" s="2" t="inlineStr">
+        <is>
+          <t>Glass Ceiling Light, Glass Pendant Light, Glass Shade</t>
+        </is>
+      </c>
+      <c r="L17" s="2" t="inlineStr">
+        <is>
+          <t>Clear Glass Pendant, Glass Lampshade, Ceiling Glass Light Fitting, Modern Glass Pendant</t>
+        </is>
+      </c>
+      <c r="M17" s="2" t="inlineStr">
+        <is>
+          <t>Clear Glass Globe Pendant Light for Kitchen Island, Vintage Glass Ceiling Shade E27, Modern Frosted Glass Hanging Light</t>
+        </is>
+      </c>
       <c r="N17" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: moonlight_retail_15.</t>
+          <t>Competitor seller: firstchoicelightingoutlet.</t>
         </is>
       </c>
     </row>
@@ -1424,32 +1424,32 @@
       <c r="B18" s="2" t="inlineStr"/>
       <c r="C18" s="2" t="inlineStr">
         <is>
-          <t>141200077246</t>
+          <t>283064879219</t>
         </is>
       </c>
       <c r="D18" s="2" t="inlineStr">
         <is>
-          <t>ElekTek</t>
+          <t>Giggi</t>
         </is>
       </c>
       <c r="E18" s="2" t="inlineStr">
         <is>
-          <t>ElekTek 3-Hook Ceiling Rose Pendant Plate Suspended Glass</t>
+          <t>Modern Chandelier Style Ceiling Pendant Light Shade K9</t>
         </is>
       </c>
       <c r="F18" s="2" t="inlineStr">
         <is>
-          <t>59+</t>
+          <t>600</t>
         </is>
       </c>
       <c r="G18" s="2" t="inlineStr">
         <is>
-          <t>GBP 17.25 to 19.99</t>
+          <t>GBP 21.99</t>
         </is>
       </c>
       <c r="H18" s="2" t="inlineStr">
         <is>
-          <t>99.9% (55.5K)</t>
+          <t>99.6% (21.9K)</t>
         </is>
       </c>
       <c r="I18" s="2" t="inlineStr">
@@ -1459,7 +1459,7 @@
       </c>
       <c r="J18" s="2" t="inlineStr">
         <is>
-          <t>Save up to 7% Multi-buy</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K18" s="2" t="inlineStr"/>
@@ -1467,7 +1467,7 @@
       <c r="M18" s="2" t="inlineStr"/>
       <c r="N18" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: buyitbetter_uk.</t>
+          <t>Competitor seller: picknmix.online.</t>
         </is>
       </c>
     </row>
@@ -1476,32 +1476,32 @@
       <c r="B19" s="2" t="inlineStr"/>
       <c r="C19" s="2" t="inlineStr">
         <is>
-          <t>356659461782</t>
+          <t>272110237788</t>
         </is>
       </c>
       <c r="D19" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>MoonLight Retail</t>
         </is>
       </c>
       <c r="E19" s="2" t="inlineStr">
         <is>
-          <t>Corinne Spiral Twill Glass Easy Fit Ceiling Pendant Light Shade</t>
+          <t>New Modern Vintage Industrial Retro Loft Glass Ceiling Lamp Shade</t>
         </is>
       </c>
       <c r="F19" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>269+</t>
         </is>
       </c>
       <c r="G19" s="2" t="inlineStr">
         <is>
-          <t>GBP 34.99 to 37.99</t>
+          <t>GBP 32.47 to 35.83</t>
         </is>
       </c>
       <c r="H19" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>100% (3.9K)</t>
         </is>
       </c>
       <c r="I19" s="2" t="inlineStr">
@@ -1511,7 +1511,7 @@
       </c>
       <c r="J19" s="2" t="inlineStr">
         <is>
-          <t>From GBP 31.49 with coupon</t>
+          <t>Save up to 5% Multi-buy</t>
         </is>
       </c>
       <c r="K19" s="2" t="inlineStr"/>
@@ -1519,45 +1519,41 @@
       <c r="M19" s="2" t="inlineStr"/>
       <c r="N19" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: moonlight_retail_15.</t>
         </is>
       </c>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="inlineStr">
-        <is>
-          <t>Spider Light</t>
-        </is>
-      </c>
+      <c r="A20" s="2" t="inlineStr"/>
       <c r="B20" s="2" t="inlineStr"/>
       <c r="C20" s="2" t="inlineStr">
         <is>
-          <t>303682816669</t>
+          <t>141200077246</t>
         </is>
       </c>
       <c r="D20" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ElekTek</t>
         </is>
       </c>
       <c r="E20" s="2" t="inlineStr">
         <is>
-          <t>Retro 4/6/8/10/12 Heads Mix-color Chandelier Spider Pendant Ceiling Light</t>
+          <t>ElekTek 3-Hook Ceiling Rose Pendant Plate Suspended Glass</t>
         </is>
       </c>
       <c r="F20" s="2" t="inlineStr">
         <is>
-          <t>67</t>
+          <t>59+</t>
         </is>
       </c>
       <c r="G20" s="2" t="inlineStr">
         <is>
-          <t>GBP 22.99 to 49.99</t>
+          <t>GBP 17.25 to 19.99</t>
         </is>
       </c>
       <c r="H20" s="2" t="inlineStr">
         <is>
-          <t>96.4% (14.7K)</t>
+          <t>99.9% (55.5K)</t>
         </is>
       </c>
       <c r="I20" s="2" t="inlineStr">
@@ -1567,27 +1563,15 @@
       </c>
       <c r="J20" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K20" s="2" t="inlineStr">
-        <is>
-          <t>Spider Light, Spider Pendant, Multi-Head Pendant Light</t>
-        </is>
-      </c>
-      <c r="L20" s="2" t="inlineStr">
-        <is>
-          <t>Sputnik Light, Multi Light Pendant, Industrial Spider Lamp, Adjustable Spider Ceiling Light</t>
-        </is>
-      </c>
-      <c r="M20" s="2" t="inlineStr">
-        <is>
-          <t>Black Multi-Head Spider Pendant Light for Living Room, Industrial Sputnik Ceiling Light 6 Head, Adjustable DIY Spider Chandelier E27</t>
-        </is>
-      </c>
+          <t>Save up to 7% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K20" s="2" t="inlineStr"/>
+      <c r="L20" s="2" t="inlineStr"/>
+      <c r="M20" s="2" t="inlineStr"/>
       <c r="N20" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: best-love2010.</t>
+          <t>Competitor seller: buyitbetter_uk.</t>
         </is>
       </c>
     </row>
@@ -1596,32 +1580,32 @@
       <c r="B21" s="2" t="inlineStr"/>
       <c r="C21" s="2" t="inlineStr">
         <is>
-          <t>303227195662</t>
+          <t>356659461782</t>
         </is>
       </c>
       <c r="D21" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E21" s="2" t="inlineStr">
         <is>
-          <t>Adjustable Pendant Light Fitting Ceiling Rose E27 Industrial Spider Hanging Lamp</t>
+          <t>Corinne Spiral Twill Glass Easy Fit Ceiling Pendant Light Shade</t>
         </is>
       </c>
       <c r="F21" s="2" t="inlineStr">
         <is>
-          <t>39</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G21" s="2" t="inlineStr">
         <is>
-          <t>GBP 13.42 to 59.92</t>
+          <t>GBP 34.99 to 37.99</t>
         </is>
       </c>
       <c r="H21" s="2" t="inlineStr">
         <is>
-          <t>99.6% (18.4K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I21" s="2" t="inlineStr">
@@ -1631,7 +1615,7 @@
       </c>
       <c r="J21" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>From GBP 31.49 with coupon</t>
         </is>
       </c>
       <c r="K21" s="2" t="inlineStr"/>
@@ -1639,16 +1623,20 @@
       <c r="M21" s="2" t="inlineStr"/>
       <c r="N21" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: nationallighting.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="inlineStr"/>
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t>Spider Light</t>
+        </is>
+      </c>
       <c r="B22" s="2" t="inlineStr"/>
       <c r="C22" s="2" t="inlineStr">
         <is>
-          <t>292861051418</t>
+          <t>303682816669</t>
         </is>
       </c>
       <c r="D22" s="2" t="inlineStr">
@@ -1658,17 +1646,17 @@
       </c>
       <c r="E22" s="2" t="inlineStr">
         <is>
-          <t>Vintage Edison Multiple Adjustable DIY Ceiling Spider Light</t>
+          <t>Retro 4/6/8/10/12 Heads Mix-color Chandelier Spider Pendant Ceiling Light</t>
         </is>
       </c>
       <c r="F22" s="2" t="inlineStr">
         <is>
-          <t>34+</t>
+          <t>67</t>
         </is>
       </c>
       <c r="G22" s="2" t="inlineStr">
         <is>
-          <t>GBP 11.99 to 21.99</t>
+          <t>GBP 22.99 to 49.99</t>
         </is>
       </c>
       <c r="H22" s="2" t="inlineStr">
@@ -1686,9 +1674,21 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K22" s="2" t="inlineStr"/>
-      <c r="L22" s="2" t="inlineStr"/>
-      <c r="M22" s="2" t="inlineStr"/>
+      <c r="K22" s="2" t="inlineStr">
+        <is>
+          <t>Spider Light, Spider Pendant, Multi-Head Pendant Light</t>
+        </is>
+      </c>
+      <c r="L22" s="2" t="inlineStr">
+        <is>
+          <t>Sputnik Light, Multi Light Pendant, Industrial Spider Lamp, Adjustable Spider Ceiling Light</t>
+        </is>
+      </c>
+      <c r="M22" s="2" t="inlineStr">
+        <is>
+          <t>Black Multi-Head Spider Pendant Light for Living Room, Industrial Sputnik Ceiling Light 6 Head, Adjustable DIY Spider Chandelier E27</t>
+        </is>
+      </c>
       <c r="N22" s="2" t="inlineStr">
         <is>
           <t>Competitor seller: best-love2010.</t>
@@ -1700,32 +1700,32 @@
       <c r="B23" s="2" t="inlineStr"/>
       <c r="C23" s="2" t="inlineStr">
         <is>
-          <t>236823130326</t>
+          <t>303227195662</t>
         </is>
       </c>
       <c r="D23" s="2" t="inlineStr">
         <is>
-          <t>ANWIO</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E23" s="2" t="inlineStr">
         <is>
-          <t>ANWIO 6 Heads Spider Light Chandelier Pendant DIY Spider Rope</t>
+          <t>Adjustable Pendant Light Fitting Ceiling Rose E27 Industrial Spider Hanging Lamp</t>
         </is>
       </c>
       <c r="F23" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>39</t>
         </is>
       </c>
       <c r="G23" s="2" t="inlineStr">
         <is>
-          <t>GBP 29.99</t>
+          <t>GBP 13.42 to 59.92</t>
         </is>
       </c>
       <c r="H23" s="2" t="inlineStr">
         <is>
-          <t>99.8% (13.4K)</t>
+          <t>99.6% (18.4K)</t>
         </is>
       </c>
       <c r="I23" s="2" t="inlineStr">
@@ -1743,45 +1743,41 @@
       <c r="M23" s="2" t="inlineStr"/>
       <c r="N23" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: wowzer-uk.</t>
+          <t>Competitor seller: nationallighting.</t>
         </is>
       </c>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Cage pendant light</t>
-        </is>
-      </c>
+      <c r="A24" s="2" t="inlineStr"/>
       <c r="B24" s="2" t="inlineStr"/>
       <c r="C24" s="2" t="inlineStr">
         <is>
-          <t>372257190104</t>
+          <t>292861051418</t>
         </is>
       </c>
       <c r="D24" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E24" s="2" t="inlineStr">
         <is>
-          <t>Ceiling Light Shade Geometric Pendant Lampshade Lamp Industrial</t>
+          <t>Vintage Edison Multiple Adjustable DIY Ceiling Spider Light</t>
         </is>
       </c>
       <c r="F24" s="2" t="inlineStr">
         <is>
-          <t>951+</t>
+          <t>34+</t>
         </is>
       </c>
       <c r="G24" s="2" t="inlineStr">
         <is>
-          <t>GBP 12.99 to 15.99</t>
+          <t>GBP 11.99 to 21.99</t>
         </is>
       </c>
       <c r="H24" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>96.4% (14.7K)</t>
         </is>
       </c>
       <c r="I24" s="2" t="inlineStr">
@@ -1791,27 +1787,15 @@
       </c>
       <c r="J24" s="2" t="inlineStr">
         <is>
-          <t>Save up to 10% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K24" s="2" t="inlineStr">
-        <is>
-          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
-        </is>
-      </c>
-      <c r="L24" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
-        </is>
-      </c>
-      <c r="M24" s="2" t="inlineStr">
-        <is>
-          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K24" s="2" t="inlineStr"/>
+      <c r="L24" s="2" t="inlineStr"/>
+      <c r="M24" s="2" t="inlineStr"/>
       <c r="N24" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: best-love2010.</t>
         </is>
       </c>
     </row>
@@ -1820,32 +1804,32 @@
       <c r="B25" s="2" t="inlineStr"/>
       <c r="C25" s="2" t="inlineStr">
         <is>
-          <t>232708905363</t>
+          <t>236823130326</t>
         </is>
       </c>
       <c r="D25" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>ANWIO</t>
         </is>
       </c>
       <c r="E25" s="2" t="inlineStr">
         <is>
-          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
+          <t>ANWIO 6 Heads Spider Light Chandelier Pendant DIY Spider Rope</t>
         </is>
       </c>
       <c r="F25" s="2" t="inlineStr">
         <is>
-          <t>289+</t>
+          <t>1</t>
         </is>
       </c>
       <c r="G25" s="2" t="inlineStr">
         <is>
-          <t>GBP 22.99 to 25.99</t>
+          <t>GBP 29.99</t>
         </is>
       </c>
       <c r="H25" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.8% (13.4K)</t>
         </is>
       </c>
       <c r="I25" s="2" t="inlineStr">
@@ -1855,7 +1839,7 @@
       </c>
       <c r="J25" s="2" t="inlineStr">
         <is>
-          <t>From GBP 20.69 with coupon</t>
+          <t>-</t>
         </is>
       </c>
       <c r="K25" s="2" t="inlineStr"/>
@@ -1863,41 +1847,45 @@
       <c r="M25" s="2" t="inlineStr"/>
       <c r="N25" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: wowzer-uk.</t>
         </is>
       </c>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="inlineStr"/>
+      <c r="A26" s="2" t="inlineStr">
+        <is>
+          <t>Cage pendant light</t>
+        </is>
+      </c>
       <c r="B26" s="2" t="inlineStr"/>
       <c r="C26" s="2" t="inlineStr">
         <is>
-          <t>131173303482</t>
+          <t>372257190104</t>
         </is>
       </c>
       <c r="D26" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E26" s="2" t="inlineStr">
         <is>
-          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
+          <t>Ceiling Light Shade Geometric Pendant Lampshade Lamp Industrial</t>
         </is>
       </c>
       <c r="F26" s="2" t="inlineStr">
         <is>
-          <t>252</t>
+          <t>951+</t>
         </is>
       </c>
       <c r="G26" s="2" t="inlineStr">
         <is>
-          <t>GBP 13.00</t>
+          <t>GBP 12.99 to 15.99</t>
         </is>
       </c>
       <c r="H26" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I26" s="2" t="inlineStr">
@@ -1907,15 +1895,27 @@
       </c>
       <c r="J26" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K26" s="2" t="inlineStr"/>
-      <c r="L26" s="2" t="inlineStr"/>
-      <c r="M26" s="2" t="inlineStr"/>
+          <t>Save up to 10% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K26" s="2" t="inlineStr">
+        <is>
+          <t>Cage Pendant Light, Cage Light, Metal Cage Pendant</t>
+        </is>
+      </c>
+      <c r="L26" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Cage Light, Wire Cage Pendant, Vintage Cage Lamp, Cage Ceiling Light</t>
+        </is>
+      </c>
+      <c r="M26" s="2" t="inlineStr">
+        <is>
+          <t>Black Metal Cage Pendant Light for Kitchen, Industrial Wire Cage Hanging Lamp E27, Vintage Cage Ceiling Light Fitting</t>
+        </is>
+      </c>
       <c r="N26" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
@@ -1924,32 +1924,32 @@
       <c r="B27" s="2" t="inlineStr"/>
       <c r="C27" s="2" t="inlineStr">
         <is>
-          <t>141264804458</t>
+          <t>232708905363</t>
         </is>
       </c>
       <c r="D27" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E27" s="2" t="inlineStr">
         <is>
-          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
+          <t>Industrial Metal Ceiling Pendant Light Shade Easy Fit</t>
         </is>
       </c>
       <c r="F27" s="2" t="inlineStr">
         <is>
-          <t>157</t>
+          <t>289+</t>
         </is>
       </c>
       <c r="G27" s="2" t="inlineStr">
         <is>
-          <t>GBP 13.00</t>
+          <t>GBP 22.99 to 25.99</t>
         </is>
       </c>
       <c r="H27" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I27" s="2" t="inlineStr">
@@ -1959,7 +1959,7 @@
       </c>
       <c r="J27" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>From GBP 20.69 with coupon</t>
         </is>
       </c>
       <c r="K27" s="2" t="inlineStr"/>
@@ -1967,7 +1967,7 @@
       <c r="M27" s="2" t="inlineStr"/>
       <c r="N27" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
@@ -1976,32 +1976,32 @@
       <c r="B28" s="2" t="inlineStr"/>
       <c r="C28" s="2" t="inlineStr">
         <is>
-          <t>262744851290</t>
+          <t>131173303482</t>
         </is>
       </c>
       <c r="D28" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Cage</t>
+          <t>Black Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
         <is>
-          <t>114</t>
+          <t>252</t>
         </is>
       </c>
       <c r="G28" s="2" t="inlineStr">
         <is>
-          <t>GBP 46.99</t>
+          <t>GBP 13.00</t>
         </is>
       </c>
       <c r="H28" s="2" t="inlineStr">
         <is>
-          <t>98.5% (15.2K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I28" s="2" t="inlineStr">
@@ -2019,45 +2019,41 @@
       <c r="M28" s="2" t="inlineStr"/>
       <c r="N28" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: sj_modern_antiques.</t>
+          <t>Competitor seller: thelampfactoryuk.</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="inlineStr">
-        <is>
-          <t>Pipe Light</t>
-        </is>
-      </c>
+      <c r="A29" s="2" t="inlineStr"/>
       <c r="B29" s="2" t="inlineStr"/>
       <c r="C29" s="2" t="inlineStr">
         <is>
-          <t>174650219163</t>
+          <t>141264804458</t>
         </is>
       </c>
       <c r="D29" s="2" t="inlineStr">
         <is>
-          <t>Stout &amp; Burg Designs</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E29" s="2" t="inlineStr">
         <is>
-          <t>Steampunk Industrial Iron Pipe Lamp/Light Socket 1-1/4 x 1/2</t>
+          <t>Bronze Wire Cage Light Shade Steel E27 Industrial Pendant</t>
         </is>
       </c>
       <c r="F29" s="2" t="inlineStr">
         <is>
-          <t>334+</t>
+          <t>157</t>
         </is>
       </c>
       <c r="G29" s="2" t="inlineStr">
         <is>
-          <t>GBP 3.18 to 10.46</t>
+          <t>GBP 13.00</t>
         </is>
       </c>
       <c r="H29" s="2" t="inlineStr">
         <is>
-          <t>99% (4.4K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I29" s="2" t="inlineStr">
@@ -2070,24 +2066,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K29" s="2" t="inlineStr">
-        <is>
-          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
-        </is>
-      </c>
-      <c r="L29" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
-        </is>
-      </c>
-      <c r="M29" s="2" t="inlineStr">
-        <is>
-          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
-        </is>
-      </c>
+      <c r="K29" s="2" t="inlineStr"/>
+      <c r="L29" s="2" t="inlineStr"/>
+      <c r="M29" s="2" t="inlineStr"/>
       <c r="N29" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: nmstoute.</t>
+          <t>Competitor seller: thelampfactoryuk.</t>
         </is>
       </c>
     </row>
@@ -2096,32 +2080,32 @@
       <c r="B30" s="2" t="inlineStr"/>
       <c r="C30" s="2" t="inlineStr">
         <is>
-          <t>333977871043</t>
+          <t>262744851290</t>
         </is>
       </c>
       <c r="D30" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E30" s="2" t="inlineStr">
         <is>
-          <t>Industrial Rustic Retro Style Pipe Light Steampunk Desk Table Lamp</t>
+          <t>Silver Industrial Ceiling Light Vintage Antique Pendant Cage</t>
         </is>
       </c>
       <c r="F30" s="2" t="inlineStr">
         <is>
-          <t>148</t>
+          <t>114</t>
         </is>
       </c>
       <c r="G30" s="2" t="inlineStr">
         <is>
-          <t>GBP 41.91</t>
+          <t>GBP 46.99</t>
         </is>
       </c>
       <c r="H30" s="2" t="inlineStr">
         <is>
-          <t>100% (1.4K)</t>
+          <t>98.5% (15.2K)</t>
         </is>
       </c>
       <c r="I30" s="2" t="inlineStr">
@@ -2139,41 +2123,45 @@
       <c r="M30" s="2" t="inlineStr"/>
       <c r="N30" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: steampunkeddesignstudio.</t>
+          <t>Competitor seller: sj_modern_antiques.</t>
         </is>
       </c>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="inlineStr"/>
+      <c r="A31" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light</t>
+        </is>
+      </c>
       <c r="B31" s="2" t="inlineStr"/>
       <c r="C31" s="2" t="inlineStr">
         <is>
-          <t>201795458338</t>
+          <t>174650219163</t>
         </is>
       </c>
       <c r="D31" s="2" t="inlineStr">
         <is>
-          <t>Mr. Willies</t>
+          <t>Stout &amp; Burg Designs</t>
         </is>
       </c>
       <c r="E31" s="2" t="inlineStr">
         <is>
-          <t>Retro Industrial Pipe Desk Table 3 bulbs steampunk edison</t>
+          <t>Steampunk Industrial Iron Pipe Lamp/Light Socket 1-1/4 x 1/2</t>
         </is>
       </c>
       <c r="F31" s="2" t="inlineStr">
         <is>
-          <t>83</t>
+          <t>334+</t>
         </is>
       </c>
       <c r="G31" s="2" t="inlineStr">
         <is>
-          <t>GBP 130.88</t>
+          <t>GBP 3.18 to 10.46</t>
         </is>
       </c>
       <c r="H31" s="2" t="inlineStr">
         <is>
-          <t>100% (882)</t>
+          <t>99% (4.4K)</t>
         </is>
       </c>
       <c r="I31" s="2" t="inlineStr">
@@ -2186,12 +2174,24 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K31" s="2" t="inlineStr"/>
-      <c r="L31" s="2" t="inlineStr"/>
-      <c r="M31" s="2" t="inlineStr"/>
+      <c r="K31" s="2" t="inlineStr">
+        <is>
+          <t>Pipe Light, Pipe Pendant Light, Steampunk Light</t>
+        </is>
+      </c>
+      <c r="L31" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Pipe Light, Steampunk Pendant, Pipe Wall Light, Water Pipe Lamp</t>
+        </is>
+      </c>
+      <c r="M31" s="2" t="inlineStr">
+        <is>
+          <t>Industrial Steampunk Pipe Pendant Light for Kitchen Island, Black Metal Pipe Ceiling Light E27, Vintage Water Pipe Wall Lamp</t>
+        </is>
+      </c>
       <c r="N31" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: mrwillieslighting.</t>
+          <t>Competitor seller: nmstoute.</t>
         </is>
       </c>
     </row>
@@ -2200,7 +2200,7 @@
       <c r="B32" s="2" t="inlineStr"/>
       <c r="C32" s="2" t="inlineStr">
         <is>
-          <t>353005301113</t>
+          <t>333977871043</t>
         </is>
       </c>
       <c r="D32" s="2" t="inlineStr">
@@ -2210,27 +2210,27 @@
       </c>
       <c r="E32" s="2" t="inlineStr">
         <is>
-          <t>Iron Vintage Steampunk Stop Valve Light Switch W/ Wire Pipe Lamp</t>
+          <t>Industrial Rustic Retro Style Pipe Light Steampunk Desk Table Lamp</t>
         </is>
       </c>
       <c r="F32" s="2" t="inlineStr">
         <is>
-          <t>77</t>
+          <t>148</t>
         </is>
       </c>
       <c r="G32" s="2" t="inlineStr">
         <is>
-          <t>GBP 16.22</t>
+          <t>GBP 41.91</t>
         </is>
       </c>
       <c r="H32" s="2" t="inlineStr">
         <is>
-          <t>99.4% (3K)</t>
+          <t>100% (1.4K)</t>
         </is>
       </c>
       <c r="I32" s="2" t="inlineStr">
         <is>
-          <t>Free postage</t>
+          <t>With postage</t>
         </is>
       </c>
       <c r="J32" s="2" t="inlineStr">
@@ -2243,7 +2243,7 @@
       <c r="M32" s="2" t="inlineStr"/>
       <c r="N32" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: happy_home_2019.</t>
+          <t>Competitor seller: steampunkeddesignstudio.</t>
         </is>
       </c>
     </row>
@@ -2252,32 +2252,32 @@
       <c r="B33" s="2" t="inlineStr"/>
       <c r="C33" s="2" t="inlineStr">
         <is>
-          <t>164791375113</t>
+          <t>201795458338</t>
         </is>
       </c>
       <c r="D33" s="2" t="inlineStr">
         <is>
-          <t>(not listed)</t>
+          <t>Mr. Willies</t>
         </is>
       </c>
       <c r="E33" s="2" t="inlineStr">
         <is>
-          <t>Retro Switch Valve Steampunk Light Industrial Pipe Table Lamp</t>
+          <t>Retro Industrial Pipe Desk Table 3 bulbs steampunk edison</t>
         </is>
       </c>
       <c r="F33" s="2" t="inlineStr">
         <is>
-          <t>25</t>
+          <t>83</t>
         </is>
       </c>
       <c r="G33" s="2" t="inlineStr">
         <is>
-          <t>GBP 10.48</t>
+          <t>GBP 130.88</t>
         </is>
       </c>
       <c r="H33" s="2" t="inlineStr">
         <is>
-          <t>99.3% (26.9K)</t>
+          <t>100% (882)</t>
         </is>
       </c>
       <c r="I33" s="2" t="inlineStr">
@@ -2295,50 +2295,46 @@
       <c r="M33" s="2" t="inlineStr"/>
       <c r="N33" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: ztt_online.</t>
+          <t>Competitor seller: mrwillieslighting.</t>
         </is>
       </c>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="inlineStr">
-        <is>
-          <t>Bulbs</t>
-        </is>
-      </c>
+      <c r="A34" s="2" t="inlineStr"/>
       <c r="B34" s="2" t="inlineStr"/>
       <c r="C34" s="2" t="inlineStr">
         <is>
-          <t>223224109836</t>
+          <t>353005301113</t>
         </is>
       </c>
       <c r="D34" s="2" t="inlineStr">
         <is>
-          <t>Auraglow</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E34" s="2" t="inlineStr">
         <is>
-          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style Decorative E27 T30 Tube</t>
+          <t>Iron Vintage Steampunk Stop Valve Light Switch W/ Wire Pipe Lamp</t>
         </is>
       </c>
       <c r="F34" s="2" t="inlineStr">
         <is>
-          <t>180</t>
+          <t>77</t>
         </is>
       </c>
       <c r="G34" s="2" t="inlineStr">
         <is>
-          <t>GBP 10.99</t>
+          <t>GBP 16.22</t>
         </is>
       </c>
       <c r="H34" s="2" t="inlineStr">
         <is>
-          <t>99.8% (188.5K)</t>
+          <t>99.4% (3K)</t>
         </is>
       </c>
       <c r="I34" s="2" t="inlineStr">
         <is>
-          <t>With postage</t>
+          <t>Free postage</t>
         </is>
       </c>
       <c r="J34" s="2" t="inlineStr">
@@ -2346,24 +2342,12 @@
           <t>-</t>
         </is>
       </c>
-      <c r="K34" s="2" t="inlineStr">
-        <is>
-          <t>LED Bulb, Filament Bulb, Light Bulb</t>
-        </is>
-      </c>
-      <c r="L34" s="2" t="inlineStr">
-        <is>
-          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
-        </is>
-      </c>
-      <c r="M34" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
-        </is>
-      </c>
+      <c r="K34" s="2" t="inlineStr"/>
+      <c r="L34" s="2" t="inlineStr"/>
+      <c r="M34" s="2" t="inlineStr"/>
       <c r="N34" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: safield-online.</t>
+          <t>Competitor seller: happy_home_2019.</t>
         </is>
       </c>
     </row>
@@ -2372,32 +2356,32 @@
       <c r="B35" s="2" t="inlineStr"/>
       <c r="C35" s="2" t="inlineStr">
         <is>
-          <t>353725905176</t>
+          <t>164791375113</t>
         </is>
       </c>
       <c r="D35" s="2" t="inlineStr">
         <is>
-          <t>Kanlux</t>
+          <t>(not listed)</t>
         </is>
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>10x EXTRA LARGE GLOBE FILAMENT E27 BULB Vintage Incandescent Edison</t>
+          <t>Retro Switch Valve Steampunk Light Industrial Pipe Table Lamp</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
         <is>
-          <t>10</t>
+          <t>25</t>
         </is>
       </c>
       <c r="G35" s="2" t="inlineStr">
         <is>
-          <t>GBP 70.94</t>
+          <t>GBP 10.48</t>
         </is>
       </c>
       <c r="H35" s="2" t="inlineStr">
         <is>
-          <t>99.7% (84.9K)</t>
+          <t>99.3% (26.9K)</t>
         </is>
       </c>
       <c r="I35" s="2" t="inlineStr">
@@ -2415,41 +2399,45 @@
       <c r="M35" s="2" t="inlineStr"/>
       <c r="N35" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: auctionzltd.</t>
+          <t>Competitor seller: ztt_online.</t>
         </is>
       </c>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="inlineStr"/>
+      <c r="A36" s="2" t="inlineStr">
+        <is>
+          <t>Bulbs</t>
+        </is>
+      </c>
       <c r="B36" s="2" t="inlineStr"/>
       <c r="C36" s="2" t="inlineStr">
         <is>
-          <t>352802795272</t>
+          <t>223224109836</t>
         </is>
       </c>
       <c r="D36" s="2" t="inlineStr">
         <is>
-          <t>ValueLights</t>
+          <t>Auraglow</t>
         </is>
       </c>
       <c r="E36" s="2" t="inlineStr">
         <is>
-          <t>Filament LED Light Bulb Decorative Vintage Edison Lightbulb</t>
+          <t>Auraglow Mysa LED Light Bulb Vintage Retro Edison Style Decorative E27 T30 Tube</t>
         </is>
       </c>
       <c r="F36" s="2" t="inlineStr">
         <is>
-          <t>102+</t>
+          <t>180</t>
         </is>
       </c>
       <c r="G36" s="2" t="inlineStr">
         <is>
-          <t>GBP 5.99 to 19.99</t>
+          <t>GBP 10.99</t>
         </is>
       </c>
       <c r="H36" s="2" t="inlineStr">
         <is>
-          <t>99.8% (685K)</t>
+          <t>99.8% (188.5K)</t>
         </is>
       </c>
       <c r="I36" s="2" t="inlineStr">
@@ -2459,15 +2447,27 @@
       </c>
       <c r="J36" s="2" t="inlineStr">
         <is>
-          <t>Save up to 15% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K36" s="2" t="inlineStr"/>
-      <c r="L36" s="2" t="inlineStr"/>
-      <c r="M36" s="2" t="inlineStr"/>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K36" s="2" t="inlineStr">
+        <is>
+          <t>LED Bulb, Filament Bulb, Light Bulb</t>
+        </is>
+      </c>
+      <c r="L36" s="2" t="inlineStr">
+        <is>
+          <t>Edison Bulb, Vintage LED Bulb, E27 Bulb, Dimmable LED Filament Bulb</t>
+        </is>
+      </c>
+      <c r="M36" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Edison LED Filament Bulb Warm White, Dimmable Squirrel Cage Light Bulb, ST64 Amber Decorative LED Bulb 4W</t>
+        </is>
+      </c>
       <c r="N36" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: value-lights.</t>
+          <t>Competitor seller: safield-online.</t>
         </is>
       </c>
     </row>
@@ -2476,32 +2476,32 @@
       <c r="B37" s="2" t="inlineStr"/>
       <c r="C37" s="2" t="inlineStr">
         <is>
-          <t>142340181955</t>
+          <t>353725905176</t>
         </is>
       </c>
       <c r="D37" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Kanlux</t>
         </is>
       </c>
       <c r="E37" s="2" t="inlineStr">
         <is>
-          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Clear Warm White Dimmable</t>
+          <t>10x EXTRA LARGE GLOBE FILAMENT E27 BULB Vintage Incandescent Edison</t>
         </is>
       </c>
       <c r="F37" s="2" t="inlineStr">
         <is>
-          <t>169</t>
+          <t>10</t>
         </is>
       </c>
       <c r="G37" s="2" t="inlineStr">
         <is>
-          <t>GBP 3.50</t>
+          <t>GBP 70.94</t>
         </is>
       </c>
       <c r="H37" s="2" t="inlineStr">
         <is>
-          <t>99.8% (22.6K)</t>
+          <t>99.7% (84.9K)</t>
         </is>
       </c>
       <c r="I37" s="2" t="inlineStr">
@@ -2519,7 +2519,7 @@
       <c r="M37" s="2" t="inlineStr"/>
       <c r="N37" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: thelampfactoryuk.</t>
+          <t>Competitor seller: auctionzltd.</t>
         </is>
       </c>
     </row>
@@ -2528,32 +2528,32 @@
       <c r="B38" s="2" t="inlineStr"/>
       <c r="C38" s="2" t="inlineStr">
         <is>
-          <t>364884514396</t>
+          <t>352802795272</t>
         </is>
       </c>
       <c r="D38" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>ValueLights</t>
         </is>
       </c>
       <c r="E38" s="2" t="inlineStr">
         <is>
-          <t>2x 4W (=33W) Vintage T30 Tube Gold LED Filament ES E27 2700K Light Bulbs</t>
+          <t>Filament LED Light Bulb Decorative Vintage Edison Lightbulb</t>
         </is>
       </c>
       <c r="F38" s="2" t="inlineStr">
         <is>
-          <t>5</t>
+          <t>102+</t>
         </is>
       </c>
       <c r="G38" s="2" t="inlineStr">
         <is>
-          <t>GBP 9.99</t>
+          <t>GBP 5.99 to 19.99</t>
         </is>
       </c>
       <c r="H38" s="2" t="inlineStr">
         <is>
-          <t>99.6% (185.3K)</t>
+          <t>99.8% (685K)</t>
         </is>
       </c>
       <c r="I38" s="2" t="inlineStr">
@@ -2563,7 +2563,7 @@
       </c>
       <c r="J38" s="2" t="inlineStr">
         <is>
-          <t>Save up to 8% Multi-buy</t>
+          <t>Save up to 15% Multi-buy</t>
         </is>
       </c>
       <c r="K38" s="2" t="inlineStr"/>
@@ -2571,45 +2571,41 @@
       <c r="M38" s="2" t="inlineStr"/>
       <c r="N38" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: dqpltd.</t>
+          <t>Competitor seller: value-lights.</t>
         </is>
       </c>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder</t>
-        </is>
-      </c>
+      <c r="A39" s="2" t="inlineStr"/>
       <c r="B39" s="2" t="inlineStr"/>
       <c r="C39" s="2" t="inlineStr">
         <is>
-          <t>396977702027</t>
+          <t>142340181955</t>
         </is>
       </c>
       <c r="D39" s="2" t="inlineStr">
         <is>
-          <t>Luxa</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E39" s="2" t="inlineStr">
         <is>
-          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose Pendant Kit</t>
+          <t>Vintage Edison Filament LED Bulb Teardrop E27 ES 4W Clear Warm White Dimmable</t>
         </is>
       </c>
       <c r="F39" s="2" t="inlineStr">
         <is>
-          <t>38</t>
+          <t>169</t>
         </is>
       </c>
       <c r="G39" s="2" t="inlineStr">
         <is>
-          <t>GBP 8.99</t>
+          <t>GBP 3.50</t>
         </is>
       </c>
       <c r="H39" s="2" t="inlineStr">
         <is>
-          <t>100% (2.5K)</t>
+          <t>99.8% (22.6K)</t>
         </is>
       </c>
       <c r="I39" s="2" t="inlineStr">
@@ -2619,27 +2615,15 @@
       </c>
       <c r="J39" s="2" t="inlineStr">
         <is>
-          <t>Save up to 5% Multi-buy</t>
-        </is>
-      </c>
-      <c r="K39" s="2" t="inlineStr">
-        <is>
-          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
-        </is>
-      </c>
-      <c r="L39" s="2" t="inlineStr">
-        <is>
-          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
-        </is>
-      </c>
-      <c r="M39" s="2" t="inlineStr">
-        <is>
-          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
-        </is>
-      </c>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K39" s="2" t="inlineStr"/>
+      <c r="L39" s="2" t="inlineStr"/>
+      <c r="M39" s="2" t="inlineStr"/>
       <c r="N39" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: gmuk.ltd.</t>
+          <t>Competitor seller: thelampfactoryuk.</t>
         </is>
       </c>
     </row>
@@ -2648,32 +2632,32 @@
       <c r="B40" s="2" t="inlineStr"/>
       <c r="C40" s="2" t="inlineStr">
         <is>
-          <t>225227368158</t>
+          <t>364884514396</t>
         </is>
       </c>
       <c r="D40" s="2" t="inlineStr">
         <is>
-          <t>Crown</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E40" s="2" t="inlineStr">
         <is>
-          <t>E27 Ceiling Rose Pendant With Tube And Lamp Holder Brass Light Fitting UK</t>
+          <t>2x 4W (=33W) Vintage T30 Tube Gold LED Filament ES E27 2700K Light Bulbs</t>
         </is>
       </c>
       <c r="F40" s="2" t="inlineStr">
         <is>
-          <t>11</t>
+          <t>5</t>
         </is>
       </c>
       <c r="G40" s="2" t="inlineStr">
         <is>
-          <t>GBP 18.85</t>
+          <t>GBP 9.99</t>
         </is>
       </c>
       <c r="H40" s="2" t="inlineStr">
         <is>
-          <t>100% (1.2K)</t>
+          <t>99.6% (185.3K)</t>
         </is>
       </c>
       <c r="I40" s="2" t="inlineStr">
@@ -2683,7 +2667,7 @@
       </c>
       <c r="J40" s="2" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Save up to 8% Multi-buy</t>
         </is>
       </c>
       <c r="K40" s="2" t="inlineStr"/>
@@ -2691,59 +2675,75 @@
       <c r="M40" s="2" t="inlineStr"/>
       <c r="N40" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: universalmerchandise4u.</t>
+          <t>Competitor seller: dqpltd.</t>
         </is>
       </c>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="inlineStr"/>
+      <c r="A41" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder</t>
+        </is>
+      </c>
       <c r="B41" s="2" t="inlineStr"/>
       <c r="C41" s="2" t="inlineStr">
         <is>
-          <t>224707047105</t>
+          <t>396977702027</t>
         </is>
       </c>
       <c r="D41" s="2" t="inlineStr">
         <is>
-          <t>Unbranded</t>
+          <t>Luxa</t>
         </is>
       </c>
       <c r="E41" s="2" t="inlineStr">
         <is>
-          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Flex Pendant Lamp Bulb Holder</t>
+          <t>Black Retro E27 Vintage Screw In Light Bulb Lamp Holder Ceiling Rose Pendant Kit</t>
         </is>
       </c>
       <c r="F41" s="2" t="inlineStr">
         <is>
-          <t>18</t>
+          <t>38</t>
         </is>
       </c>
       <c r="G41" s="2" t="inlineStr">
         <is>
-          <t>GBP 10.59</t>
+          <t>GBP 8.99</t>
         </is>
       </c>
       <c r="H41" s="2" t="inlineStr">
         <is>
-          <t>99.6% (2.9K)</t>
+          <t>100% (2.5K)</t>
         </is>
       </c>
       <c r="I41" s="2" t="inlineStr">
         <is>
-          <t>Free postage</t>
+          <t>With postage</t>
         </is>
       </c>
       <c r="J41" s="2" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="K41" s="2" t="inlineStr"/>
-      <c r="L41" s="2" t="inlineStr"/>
-      <c r="M41" s="2" t="inlineStr"/>
+          <t>Save up to 5% Multi-buy</t>
+        </is>
+      </c>
+      <c r="K41" s="2" t="inlineStr">
+        <is>
+          <t>Lamp Holder, Bulb Holder, E27 Holder</t>
+        </is>
+      </c>
+      <c r="L41" s="2" t="inlineStr">
+        <is>
+          <t>Ceiling Rose Lamp Holder, Pendant Lamp Holder, Bakelite Bulb Holder, E27 Fitting</t>
+        </is>
+      </c>
+      <c r="M41" s="2" t="inlineStr">
+        <is>
+          <t>E27 Vintage Bakelite Pendant Lamp Holder with Cord Grip, Ceiling Rose Bulb Holder Kit, Screw E27 Fitting with Switch</t>
+        </is>
+      </c>
       <c r="N41" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: yuki-store-2020.</t>
+          <t>Competitor seller: gmuk.ltd.</t>
         </is>
       </c>
     </row>
@@ -2752,32 +2752,32 @@
       <c r="B42" s="2" t="inlineStr"/>
       <c r="C42" s="2" t="inlineStr">
         <is>
-          <t>274419951502</t>
+          <t>225227368158</t>
         </is>
       </c>
       <c r="D42" s="2" t="inlineStr">
         <is>
-          <t>Crown Lighting</t>
+          <t>Crown</t>
         </is>
       </c>
       <c r="E42" s="2" t="inlineStr">
         <is>
-          <t>E27 Modern Ceiling Rose Pendant With Tube And Lamp Holder Fitting</t>
+          <t>E27 Ceiling Rose Pendant With Tube And Lamp Holder Brass Light Fitting UK</t>
         </is>
       </c>
       <c r="F42" s="2" t="inlineStr">
         <is>
-          <t>2</t>
+          <t>11</t>
         </is>
       </c>
       <c r="G42" s="2" t="inlineStr">
         <is>
-          <t>GBP 24.95</t>
+          <t>GBP 18.85</t>
         </is>
       </c>
       <c r="H42" s="2" t="inlineStr">
         <is>
-          <t>100% (8.5K)</t>
+          <t>100% (1.2K)</t>
         </is>
       </c>
       <c r="I42" s="2" t="inlineStr">
@@ -2795,7 +2795,7 @@
       <c r="M42" s="2" t="inlineStr"/>
       <c r="N42" s="2" t="inlineStr">
         <is>
-          <t>Competitor seller: bandhstore.</t>
+          <t>Competitor seller: universalmerchandise4u.</t>
         </is>
       </c>
     </row>
@@ -2804,37 +2804,37 @@
       <c r="B43" s="2" t="inlineStr"/>
       <c r="C43" s="2" t="inlineStr">
         <is>
-          <t>184848546669</t>
+          <t>224707047105</t>
         </is>
       </c>
       <c r="D43" s="2" t="inlineStr">
         <is>
-          <t>Knightsbridge</t>
+          <t>Unbranded</t>
         </is>
       </c>
       <c r="E43" s="2" t="inlineStr">
         <is>
-          <t>ES E27 Screw In Bulb Lamp Matt White Pendant Set Lampholder Ceiling Rose</t>
+          <t>E27 Ceiling Rose Light Fitting Vintage Industrial Flex Pendant Lamp Bulb Holder</t>
         </is>
       </c>
       <c r="F43" s="2" t="inlineStr">
         <is>
-          <t>22</t>
+          <t>18</t>
         </is>
       </c>
       <c r="G43" s="2" t="inlineStr">
         <is>
-          <t>GBP 18.99</t>
+          <t>GBP 10.59</t>
         </is>
       </c>
       <c r="H43" s="2" t="inlineStr">
         <is>
-          <t>99.9% (44.1K)</t>
+          <t>99.6% (2.9K)</t>
         </is>
       </c>
       <c r="I43" s="2" t="inlineStr">
         <is>
-          <t>With postage</t>
+          <t>Free postage</t>
         </is>
       </c>
       <c r="J43" s="2" t="inlineStr">
@@ -2847,6 +2847,110 @@
       <c r="M43" s="2" t="inlineStr"/>
       <c r="N43" s="2" t="inlineStr">
         <is>
+          <t>Competitor seller: yuki-store-2020.</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="2" t="inlineStr"/>
+      <c r="B44" s="2" t="inlineStr"/>
+      <c r="C44" s="2" t="inlineStr">
+        <is>
+          <t>274419951502</t>
+        </is>
+      </c>
+      <c r="D44" s="2" t="inlineStr">
+        <is>
+          <t>Crown Lighting</t>
+        </is>
+      </c>
+      <c r="E44" s="2" t="inlineStr">
+        <is>
+          <t>E27 Modern Ceiling Rose Pendant With Tube And Lamp Holder Fitting</t>
+        </is>
+      </c>
+      <c r="F44" s="2" t="inlineStr">
+        <is>
+          <t>2</t>
+        </is>
+      </c>
+      <c r="G44" s="2" t="inlineStr">
+        <is>
+          <t>GBP 24.95</t>
+        </is>
+      </c>
+      <c r="H44" s="2" t="inlineStr">
+        <is>
+          <t>100% (8.5K)</t>
+        </is>
+      </c>
+      <c r="I44" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K44" s="2" t="inlineStr"/>
+      <c r="L44" s="2" t="inlineStr"/>
+      <c r="M44" s="2" t="inlineStr"/>
+      <c r="N44" s="2" t="inlineStr">
+        <is>
+          <t>Competitor seller: bandhstore.</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="2" t="inlineStr"/>
+      <c r="B45" s="2" t="inlineStr"/>
+      <c r="C45" s="2" t="inlineStr">
+        <is>
+          <t>184848546669</t>
+        </is>
+      </c>
+      <c r="D45" s="2" t="inlineStr">
+        <is>
+          <t>Knightsbridge</t>
+        </is>
+      </c>
+      <c r="E45" s="2" t="inlineStr">
+        <is>
+          <t>ES E27 Screw In Bulb Lamp Matt White Pendant Set Lampholder Ceiling Rose</t>
+        </is>
+      </c>
+      <c r="F45" s="2" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="G45" s="2" t="inlineStr">
+        <is>
+          <t>GBP 18.99</t>
+        </is>
+      </c>
+      <c r="H45" s="2" t="inlineStr">
+        <is>
+          <t>99.9% (44.1K)</t>
+        </is>
+      </c>
+      <c r="I45" s="2" t="inlineStr">
+        <is>
+          <t>With postage</t>
+        </is>
+      </c>
+      <c r="J45" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="K45" s="2" t="inlineStr"/>
+      <c r="L45" s="2" t="inlineStr"/>
+      <c r="M45" s="2" t="inlineStr"/>
+      <c r="N45" s="2" t="inlineStr">
+        <is>
           <t>Competitor seller: colchester-electrical-wholesale.</t>
         </is>
       </c>

</xml_diff>